<commit_message>
Fixed metadata family - which rows to read
</commit_message>
<xml_diff>
--- a/notebook/locations.xlsx
+++ b/notebook/locations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V247"/>
+  <dimension ref="A1:AB269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,36 @@
           <t>de.wikipedia.org</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>www.stolpersteine-berlin.de</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>apps.bundesarchiv.de</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>collections.yadvashem.org</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>commons.wikimedia.org</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>atom.lib.uct.ac.za</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>www.lotta-magazin.de</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2867,6 +2897,11 @@
           <t>11 giessen marktplatz</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Marktplatz 11</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr">
         <is>
           <t>50.58727</t>
@@ -4514,6 +4549,16 @@
           <t>GO</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2944820/breidenbach.html</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q564579</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4721,6 +4766,16 @@
           <t>GO</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2825297/stuttgart.html</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q1022</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5240,6 +5295,16 @@
           <t>GO</t>
         </is>
       </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/12217751/theresienstadt-concentration-camp-and-ghetto.html</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q160175</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6785,6 +6850,523 @@
         </is>
       </c>
     </row>
+    <row r="248"/>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Steinstraße 19,</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>19 steinstraße</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Wullenweberstraße 11, Berlin-Moabit</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>11 berlinmoabit wullenweberstraße</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>erinnerungsort</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2950159</t>
+        </is>
+      </c>
+      <c r="W250" t="inlineStr">
+        <is>
+          <t>https://www.stolpersteine-berlin.de/de/wullenweberstr/11/auguste-stern</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Wölfersheim</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>wölfersheim</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2806852/woelfersheim.html</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q634098</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Koblenz</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>koblenz</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>erinnerungsort</t>
+        </is>
+      </c>
+      <c r="X252" t="inlineStr">
+        <is>
+          <t>https://apps.bundesarchiv.de/gedenkbuch/de976422</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Yad Vashem</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>vashem yad</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>erinnerungsort</t>
+        </is>
+      </c>
+      <c r="Y253" t="inlineStr">
+        <is>
+          <t>https://collections.yadvashem.org/en/names/13219727</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Baiertal</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>baiertal</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2953189/baiertal.html</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q7904</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Lollar</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>lollar</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/6557780</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>states united</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>neue_heimat</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/6252001/united-states.html</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q30</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Berdytschiw</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>berdytschiw</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/712441/berdychiv.html</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q7904</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Oberhessen</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>oberhessen</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q15837262</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Marktplatz 11</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>11 marktplatz</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>https://www.giessen.de/index.php?ModID=7&amp;FID=2874.2939.1&amp;object=tx%7C2874.2939.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Walltorstraße 48</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>48 walltorstraße</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>ort_der_zeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>KZ Buchenwald</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>buchenwald kz</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Buchenwald</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>ort_der_zeit</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/8644023/konzentrationslager-buchenwald.html</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q152802</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Darmstadt</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>darmstadt</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>verkehrsmittel</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2938913/darmstadt.html</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q2973</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Treblinka (Vernichtungslager)</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>treblinka vernichtungslager</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>ort_der_zeit</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/756807/treblinka.html</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q152010</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Gießen Marktplatz 15</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>15 gießen marktplatz</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Gießen</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>erinnerungsort</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2920512</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>https://www.giessen.de/Erleben/Über-Gießen/Stolpersteine/Marktplatz-15</t>
+        </is>
+      </c>
+      <c r="Z264" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Stolperstein_Gießen_Marktplatz_15_Esther_Stern.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Sennfeld (Adelsheim)</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>adelsheim sennfeld</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Sennfeld</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>https://www.geonames.org/2833011/sennfeld.html</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q14531586</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>aus Gießen nach Palästina</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>aus gießen nach palästina</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Gießen</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>verkehrsmittel</t>
+        </is>
+      </c>
+      <c r="AA266" t="inlineStr">
+        <is>
+          <t>https://atom.lib.uct.ac.za/uploads/r/university-of-cape-town-libraries-special-collections/a/3/c/a3cc8572f727d61327e4f929a86fc91c339c13cc41721aa18c8f158e13678891/mss_sahgf_schragenheim_publications_025_1-20.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Gießen Schillerschule (Volksschule)</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>gießen schillerschule volksschule</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Gießen</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>alte_heimat</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>https://www.giessen.de/index.php?ModID=7&amp;FID=2874.2967.1&amp;object=tx%2C2874.2967.1</t>
+        </is>
+      </c>
+      <c r="V267" t="inlineStr">
+        <is>
+          <t>https://de.wikipedia.org/wiki/Datei:Stolperstein_Gießen_Nordanlage_Esther_Stern.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Esther-Stern-Platz Gießen</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>esthersternplatz gießen</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Gießen</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>erinnerungsort</t>
+        </is>
+      </c>
+      <c r="AB268" t="inlineStr">
+        <is>
+          <t>https://www.lotta-magazin.de/ausgabe/1/den-ermordeten-menschen-ein-gesicht-geben/</t>
+        </is>
+      </c>
+    </row>
+    <row r="269"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added person to events table in location detail page
</commit_message>
<xml_diff>
--- a/notebook/locations.xlsx
+++ b/notebook/locations.xlsx
@@ -1113,12 +1113,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>GO - geographischer Ort</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; India &gt; Maharashtra &gt; Mumbai</t>
+          <t>GO – geographischer Ort</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2168,12 +2168,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Campello sul Clitunno</t>
+          <t>GO - geographischer Ort</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Italia &gt; Umbria &gt; Campello sul Clitunno</t>
+          <t>GO – geographischer Ort</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2309,12 +2309,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Kehl</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Deutschland &gt; Kehl</t>
+          <t>GO – geographischer Ort &gt; Deutschland</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ein HaNetziv</t>
+          <t>Kibbuz</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Palästina – Israel &gt; Kibbuz &gt; Ein HaNetziv</t>
+          <t>GO – geographischer Ort &gt; Palästina – Israel &gt; Kibbuz</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2438,12 +2438,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Kibbuz Rodges</t>
+          <t>Kibbuz</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Palästina – Israel &gt; Kibbuz &gt; Kibbuz Rodges</t>
+          <t>GO – geographischer Ort &gt; Palästina – Israel &gt; Kibbuz</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2476,12 +2476,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tirat Tsvi</t>
+          <t>Kibbuz</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Palästina – Israel &gt; Kibbuz &gt; Tirat Tsvi</t>
+          <t>GO – geographischer Ort &gt; Palästina – Israel &gt; Kibbuz</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3047,12 +3047,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Poznan</t>
+          <t>Polen</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Polska &gt; województwo wielkopolskie &gt; Poznań</t>
+          <t>GO – geographischer Ort &gt; Polen</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3298,12 +3298,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Sennfeld</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Deutschland &gt; Gießen &gt; Sennfeld</t>
+          <t>GO – geographischer Ort &gt; Deutschland</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3346,12 +3346,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>GO - geographischer Ort</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Singapore &gt; Singapore</t>
+          <t>GO – geographischer Ort</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3644,12 +3644,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Wolka Okraglik</t>
+          <t>Polen</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Polska &gt; województwo mazowieckie &gt; gmina Kosów Lacki &gt; Wólka Okrąglik</t>
+          <t>GO – geographischer Ort &gt; Polen</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3802,10 +3802,10 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>50.5895607</v>
+        <v>50.589967</v>
       </c>
       <c r="G62" t="n">
-        <v>8.6775827</v>
+        <v>8.6783959</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -4086,12 +4086,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Kannavia</t>
+          <t>GO - geographischer Ort</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GO – geographischer Ort &gt; Κύπρος - Kıbrıs &gt; Κύπρος &gt; Καννάβια &gt; Kannavia</t>
+          <t>GO – geographischer Ort</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">

</xml_diff>